<commit_message>
The AI-CAIQ workbook was invalid: 'OSP' is not an ownership value
Caught while assessing a second subject against the same renderer. The
eleven real SSRM dropdown strings are "Owned by CSP/MP/OSP/AP/AIC",
"Shared ...", "Not Determined" -- and this workbook carried bare 'OSP',
which CSA's own dropdown validation rejects.

It shipped because fill_ai_caiq.py does not check ownership values against
the template despite its README claiming it hard-errors on anything else
(moonsoup/rockin-robin#18). Re-rendered and confirmed with
rich-text/scripts/verify_ai_caiq_workbook.py: only C:F changed, vocabulary
intact.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jf6LUfPUm4H3UM3dLrwBh4
</commit_message>
<xml_diff>
--- a/docs/ai-caiq/AI-CAIQ-spindlebox-v1.1.0.xlsx
+++ b/docs/ai-caiq/AI-CAIQ-spindlebox-v1.1.0.xlsx
@@ -2306,7 +2306,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="D46" s="18" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E46" s="18" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D48" s="18" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E48" s="18" t="inlineStr">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="D219" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
@@ -8852,7 +8852,7 @@
       </c>
       <c r="D220" s="18" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E220" s="18" t="inlineStr">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="D229" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E229" s="14" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="D231" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E231" s="14" t="inlineStr">
@@ -10697,7 +10697,7 @@
       </c>
       <c r="D282" s="18" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E282" s="18" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="D283" s="14" t="inlineStr">
         <is>
-          <t>OSP</t>
+          <t>Owned by OSP</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">

</xml_diff>